<commit_message>
Complete work flow of ecommerce website
</commit_message>
<xml_diff>
--- a/src/test/resources/excel/testData.xlsx
+++ b/src/test/resources/excel/testData.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\premk\eclipse-workspace\SauceDemoFramework\src\test\resources\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F3EEBFA-47B0-4E25-9FE7-C119ED444A87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C69071D-6BD0-4236-B05E-1ED725911719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9360" yWindow="504" windowWidth="11628" windowHeight="11736" xr2:uid="{B0716547-B3AF-484E-A127-FF93F9BD8DF9}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="loginTest" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,6 +31,26 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>standard_user</t>
+  </si>
+  <si>
+    <t>secret_sauce</t>
+  </si>
+  <si>
+    <t>locked_out_user</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -380,9 +400,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B13749F1-7146-470C-9E01-22AD72143D65}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Logic seperated from main test method. code optimized
</commit_message>
<xml_diff>
--- a/src/test/resources/excel/testData.xlsx
+++ b/src/test/resources/excel/testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\premk\eclipse-workspace\SauceDemoFramework\src\test\resources\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C69071D-6BD0-4236-B05E-1ED725911719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02640569-2BFC-492B-BCEE-7264374D5468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9360" yWindow="504" windowWidth="11628" windowHeight="11736" xr2:uid="{B0716547-B3AF-484E-A127-FF93F9BD8DF9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B0716547-B3AF-484E-A127-FF93F9BD8DF9}"/>
   </bookViews>
   <sheets>
     <sheet name="loginTest" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>user</t>
   </si>
@@ -49,6 +49,15 @@
   </si>
   <si>
     <t>locked_out_user</t>
+  </si>
+  <si>
+    <t>productName</t>
+  </si>
+  <si>
+    <t>Sauce Labs Bolt T-Shirt</t>
+  </si>
+  <si>
+    <t>Sauce Labs Backpack,Sauce Labs Bolt T-Shirt,Sauce Labs Fleece Jacket</t>
   </si>
 </sst>
 </file>
@@ -400,31 +409,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B13749F1-7146-470C-9E01-22AD72143D65}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>